<commit_message>
Rewrite two summaries, correct one sentiment
</commit_message>
<xml_diff>
--- a/templates/HR_Intelligence_Master_Tracker.xlsx
+++ b/templates/HR_Intelligence_Master_Tracker.xlsx
@@ -940,75 +940,247 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>M-20260808-001</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>46242</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>RK World Infocom</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Culture</t>
+        </is>
+      </c>
       <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n"/>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>good company to work for</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Reviews/Employee-Review-Rk-Worldinfocom-E8268877-RVW105157672.htm</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Current Employee</t>
+        </is>
+      </c>
       <c r="N2" s="5" t="n"/>
-      <c r="O2" s="14" t="n"/>
+      <c r="O2" s="14" t="n">
+        <v>5</v>
+      </c>
       <c r="P2" s="5" t="n"/>
-      <c r="Q2" s="5" t="n"/>
-      <c r="R2" s="5" t="n"/>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="S2" s="5" t="n"/>
-      <c r="T2" s="5" t="n"/>
-      <c r="U2" s="5" t="n"/>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
       <c r="V2" s="5" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>M-20260829-001</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>46268</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>46263</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>RK Group</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>AmbitionBox</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>AmbitionBox</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Management | Culture</t>
+        </is>
+      </c>
       <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>There is big politics inside the company old people don't want work according to new guys they always pinch to director or uppper lavel management.7 days (Flexible Timings), This job involves Travel Within Country, Travel Within City.</t>
+        </is>
+      </c>
       <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="N3" s="5" t="n"/>
-      <c r="O3" s="14" t="n"/>
+      <c r="O3" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="P3" s="5" t="n"/>
-      <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="S3" s="5" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="U3" s="5" t="n"/>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
       <c r="V3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>M-20260905-001</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>46275</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>46270</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>RK World Infocom</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>AmbitionBox</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>AmbitionBox</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Culture | Appraisals</t>
+        </is>
+      </c>
       <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Team Outing, Supportive team members,Salary way below market standard, no promotions,5 days (Strict Timings), This is a desk job, Occasional overtime</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
       <c r="N4" s="5" t="n"/>
-      <c r="O4" s="14" t="n"/>
+      <c r="O4" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
       <c r="V4" s="5" t="n"/>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Correct RK Group's AmbitionBox baseline to all locations
The first reading was the Bengaluru view: 2.70 across 27 reviews. The
company-wide figure is 3.30 across 151. The location dropdown confirmed it
- Bengaluru shows exactly 27, the number that had been recorded as the
whole company.

Left uncorrected, next Friday's comparison against a real all-locations
count would have reported roughly +124 new reviews, all of which had been
there for months.

The sub-scores are cleared rather than kept. They were read off the
Bengaluru view too, and beside an all-locations headline they would read as
company-wide figures. The notes keep what the mistake revealed: Bengaluru
rates the group 0.6 lower than the rest of India, and the location split is
New Delhi 39, Bengaluru 27, Mumbai 6, Ahmedabad 5, Hyderabad 4, Lucknow 4,
Daman & Diu 3.

Glassdoor still to correct.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7dEPWfmEHdt3PdTUiNh1J
</commit_message>
<xml_diff>
--- a/templates/HR_Intelligence_Master_Tracker.xlsx
+++ b/templates/HR_Intelligence_Master_Tracker.xlsx
@@ -1055,7 +1055,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -1066,13 +1066,17 @@
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>There is big politics inside the company old people don't want work according to new guys they always pinch to director or uppper lavel management.7 days (Flexible Timings), This job involves Travel Within Country, Travel Within City.</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="n"/>
+          <t>Describes internal politics, says longer-serving staff escalate to directors rather than work with newer employees</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ambitionbox.com/reviews/r-dot-k-dot-group-reviews</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="N3" s="5" t="n"/>
@@ -1106,7 +1110,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>M-20260905-001</t>
+          <t>M-20260905-002</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
@@ -1140,19 +1144,23 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Culture | Appraisals</t>
+          <t>Salary &amp; Appraisals | Growth | Culture</t>
         </is>
       </c>
       <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Team Outing, Supportive team members,Salary way below market standard, no promotions,5 days (Strict Timings), This is a desk job, Occasional overtime</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n"/>
+          <t>Praises supportive team and outings, says salary is well below market with no promotions</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ambitionbox.com/reviews/r-k-world-infocom-reviews</t>
+        </is>
+      </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Current Employee</t>
         </is>
       </c>
       <c r="N4" s="5" t="n"/>
@@ -13972,27 +13980,17 @@
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>27</v>
+        <v>151</v>
       </c>
       <c r="E2" s="15" t="n"/>
-      <c r="F2" s="7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>2.1</v>
-      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
           <t>https://www.ambitionbox.com/reviews/r-dot-k-dot-group-reviews</t>
@@ -14000,7 +13998,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>SCOPE: Bengaluru-filtered, not all locations. GENDER SPLIT: women 1.7 (7 reviews) vs men 3.5 (19) - a 1.8 point gap. Skill Development 2.3.</t>
+          <t>ALL LOCATIONS, corrected 2026-09-22. The first reading was the Bengaluru view: 2.70 across 27 reviews, against 3.30 across 151 company-wide - Bengaluru rates the group 0.6 lower than the rest of India. Locations: New Delhi 39, Bengaluru 27, Mumbai 6, Ahmedabad 5, Hyderabad 4, Lucknow 4, Daman &amp; Diu 3, others. Sub-scores cleared: they were Bengaluru-only and would have read as company-wide.</t>
         </is>
       </c>
       <c r="M2" s="7" t="n">

</xml_diff>

<commit_message>
Correct RK Group's Glassdoor baseline to all locations
3.60 across 16 reviews with 56% recommend was the Bangalore view.
Company-wide is 3.70 across 30, 64% recommend, 65% positive outlook.

With AmbitionBox corrected in the previous commit, all seven rating
snapshots now describe the population they claim to. The same city is the
weaker half on both platforms - Bengaluru 2.70 against 3.30 on AmbitionBox,
Bangalore 3.60 against 3.70 on Glassdoor - which is a finding the original
error would have buried by presenting it as the company figure.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7dEPWfmEHdt3PdTUiNh1J
</commit_message>
<xml_diff>
--- a/templates/HR_Intelligence_Master_Tracker.xlsx
+++ b/templates/HR_Intelligence_Master_Tracker.xlsx
@@ -14002,13 +14002,13 @@
         </is>
       </c>
       <c r="M2" s="7" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="N2" s="15" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="O2" s="15" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="7" t="n"/>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>SCOPE: Bangalore-filtered view only, not all locations - 16 reviews is the Bangalore subset. 69% positive business outlook. Glassdoor classifies RK Group as Manufacturing; industry average 3.5. All-locations figure still needed.</t>
+          <t>ALL LOCATIONS, corrected 2026-09-22. The first reading was the Bangalore view: 3.60 across 16 reviews, 56% recommend. Company-wide is 3.70 across 30, 64% recommend, 65% positive business outlook - so Bangalore is the weaker half on Glassdoor too, matching AmbitionBox. Glassdoor classifies RK Group as Manufacturing; industry average 3.5. Employer Profile NOT claimed.</t>
         </is>
       </c>
       <c r="X2" s="6" t="n">

</xml_diff>

<commit_message>
Regenerate the tracking workbook from the merged data
Rebuilt after the merge so the file carries both halves: the three
back-read reviews and RK Group's corrected all-locations ratings. The
version before the merge had the reviews but the old Bengaluru figures.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7dEPWfmEHdt3PdTUiNh1J
</commit_message>
<xml_diff>
--- a/templates/HR_Intelligence_Master_Tracker.xlsx
+++ b/templates/HR_Intelligence_Master_Tracker.xlsx
@@ -13980,27 +13980,17 @@
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>27</v>
+        <v>151</v>
       </c>
       <c r="E2" s="15" t="n"/>
-      <c r="F2" s="7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>2.1</v>
-      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
           <t>https://www.ambitionbox.com/reviews/r-dot-k-dot-group-reviews</t>
@@ -14008,17 +13998,17 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>SCOPE: Bengaluru-filtered, not all locations. GENDER SPLIT: women 1.7 (7 reviews) vs men 3.5 (19) - a 1.8 point gap. Skill Development 2.3.</t>
+          <t>ALL LOCATIONS, corrected 2026-09-22. The first reading was the Bengaluru view: 2.70 across 27 reviews, against 3.30 across 151 company-wide - Bengaluru rates the group 0.6 lower than the rest of India. Locations: New Delhi 39, Bengaluru 27, Mumbai 6, Ahmedabad 5, Hyderabad 4, Lucknow 4, Daman &amp; Diu 3, others. Sub-scores cleared: they were Bengaluru-only and would have read as company-wide.</t>
         </is>
       </c>
       <c r="M2" s="7" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="N2" s="15" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="O2" s="15" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="7" t="n"/>
@@ -14033,7 +14023,7 @@
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>SCOPE: Bangalore-filtered view only, not all locations - 16 reviews is the Bangalore subset. 69% positive business outlook. Glassdoor classifies RK Group as Manufacturing; industry average 3.5. All-locations figure still needed.</t>
+          <t>ALL LOCATIONS, corrected 2026-09-22. The first reading was the Bangalore view: 3.60 across 16 reviews, 56% recommend. Company-wide is 3.70 across 30, 64% recommend, 65% positive business outlook - so Bangalore is the weaker half on Glassdoor too, matching AmbitionBox. Glassdoor classifies RK Group as Manufacturing; industry average 3.5. Employer Profile NOT claimed.</t>
         </is>
       </c>
       <c r="X2" s="6" t="n">

</xml_diff>